<commit_message>
适度分包 internal/pdfenc+ooxml,examples 收录真实文档,README 增加与 Python Docling 的性能与能力对比
- 分包:根包保留公共 API 与解析编排;PDF 字节编码层(ToUnicode/
  CMap/SFNT 恢复、JPX/JBIG2 解码、软蒙版 alpha)下沉 internal/pdfenc,
  Strict OOXML 归一化下沉 internal/ooxml;跨包符号导出并保持 API
  表面不外泄(internal 对模块外不可见)
- examples:支持每目录多组样例对照;收录真实文档——学术论文 PDF
  (schmager-plateau10,源自 pdfcpu testdata)与业务透视工作簿
  (Book1.xlsx,源自 excelize testdata),expected.md 同步生成
- README 双语重写:参考 Docling 官方风格,新增 Why docparse 现代
  混合架构叙事、同机实测性能对比(纯 Go 快 34~153 倍,Mermaid 柱状图)、
  与 Python Docling 的解析能力矩阵、分包后目录结构
</commit_message>
<xml_diff>
--- a/examples/xlsx/sample.xlsx
+++ b/examples/xlsx/sample.xlsx
@@ -16,31 +16,31 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
+    <t>M-1002</t>
+  </si>
+  <si>
+    <t>电流互感器</t>
+  </si>
+  <si>
+    <t>物料编码</t>
+  </si>
+  <si>
+    <t>物料名称</t>
+  </si>
+  <si>
+    <t>库存数量</t>
+  </si>
+  <si>
+    <t>温湿度传感器</t>
+  </si>
+  <si>
+    <t>边缘网关</t>
+  </si>
+  <si>
+    <t>M-1003</t>
+  </si>
+  <si>
     <t>M-1001</t>
-  </si>
-  <si>
-    <t>库存数量</t>
-  </si>
-  <si>
-    <t>温湿度传感器</t>
-  </si>
-  <si>
-    <t>M-1002</t>
-  </si>
-  <si>
-    <t>边缘网关</t>
-  </si>
-  <si>
-    <t>M-1003</t>
-  </si>
-  <si>
-    <t>电流互感器</t>
-  </si>
-  <si>
-    <t>物料编码</t>
-  </si>
-  <si>
-    <t>物料名称</t>
   </si>
 </sst>
 </file>
@@ -349,21 +349,21 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C2">
         <v>120</v>
@@ -371,10 +371,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C3">
         <v>35</v>
@@ -382,10 +382,10 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C4">
         <v>480</v>

</xml_diff>